<commit_message>
fix: treat current_team=--- as retired in data and code
- player_status_all.csv: 11 rows with current_team=--- corrected to
  is_retired=yes and current_team empty
- merge_player_data.py: add guard at merge time to auto-fix any future
  --- values before they propagate downstream

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/data/premier_league_players_merged_final.xlsx
+++ b/backend/data/premier_league_players_merged_final.xlsx
@@ -1155,14 +1155,10 @@
       <c r="AB7" t="inlineStr"/>
       <c r="AC7" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AD7" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AD7" t="inlineStr"/>
       <c r="AE7" t="inlineStr">
         <is>
           <t>Leeds United;Everton;Newcastle United;Bolton Wanderers</t>
@@ -7673,14 +7669,10 @@
       <c r="AB80" t="inlineStr"/>
       <c r="AC80" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AD80" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AD80" t="inlineStr"/>
       <c r="AE80" t="inlineStr">
         <is>
           <t>Aston Villa;Middlesbrough</t>
@@ -28889,14 +28881,10 @@
       <c r="AB342" t="inlineStr"/>
       <c r="AC342" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AD342" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AD342" t="inlineStr"/>
       <c r="AE342" t="inlineStr">
         <is>
           <t>Bolton Wanderers</t>
@@ -36039,14 +36027,10 @@
       <c r="AB436" t="inlineStr"/>
       <c r="AC436" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="AD436" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AD436" t="inlineStr"/>
       <c r="AE436" t="inlineStr">
         <is>
           <t>Nottingham Forest;Sheffield Wednesday;Charlton Athletic;Ipswich Town</t>

</xml_diff>